<commit_message>
feat: update logbook with new entries and revisions
</commit_message>
<xml_diff>
--- a/docs/logbook.xlsx
+++ b/docs/logbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\01_Projects\EPITA\RetroHub\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A25E1FFA-9E51-454B-AE45-987180FA3284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BADB800-E234-4B5B-8373-8901A277C2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{8F73FF81-C54F-4E0C-9038-545D5E42BA1D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37710" windowHeight="21840" xr2:uid="{8F73FF81-C54F-4E0C-9038-545D5E42BA1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -20,21 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="52">
   <si>
     <t>Date</t>
   </si>
@@ -104,13 +95,112 @@
     <t>Documentation principale terminée.
 Toutes les tâches sont finies.
 Les tests ne sont pas encore faits.</t>
+  </si>
+  <si>
+    <t>J’ai ajouté Docker et MongoDB</t>
+  </si>
+  <si>
+    <t>14/01/2026</t>
+  </si>
+  <si>
+    <t>15/01/2026</t>
+  </si>
+  <si>
+    <t>J’ai amélioré le style du site</t>
+  </si>
+  <si>
+    <t>16/01/2026</t>
+  </si>
+  <si>
+    <t>J’ai conteneurisé l’application</t>
+  </si>
+  <si>
+    <t>Application complète lancée avec Docker.</t>
+  </si>
+  <si>
+    <t>17/01/2026</t>
+  </si>
+  <si>
+    <t>J’ai corrigé le proxy API</t>
+  </si>
+  <si>
+    <t>19/01/2026</t>
+  </si>
+  <si>
+    <t>J’ai ajouté des données de test</t>
+  </si>
+  <si>
+    <t>J’ai amélioré le panneau admin</t>
+  </si>
+  <si>
+    <t>20/01/2026</t>
+  </si>
+  <si>
+    <t>21/01/2026</t>
+  </si>
+  <si>
+    <t>Docker Compose configuré avec MongoDB et Mongo Express.</t>
+  </si>
+  <si>
+    <t>J’ai amélioré la base de données</t>
+  </si>
+  <si>
+    <t>Vérifications de connexion MongoDB ajoutées. Scripts Docker améliorés.</t>
+  </si>
+  <si>
+    <t>J’ai créé le logbook du projet</t>
+  </si>
+  <si>
+    <t>Fichier logbook ajouté et structuré.</t>
+  </si>
+  <si>
+    <t>J’ai amélioré l’interface admin</t>
+  </si>
+  <si>
+    <t>Gestion des erreurs et formulaires améliorés.</t>
+  </si>
+  <si>
+    <t>Thème, header et navigation mis à jour.</t>
+  </si>
+  <si>
+    <t>J’ai intégré le chat AI</t>
+  </si>
+  <si>
+    <t>Fonctionnalité de chat AI ajoutée au projet.</t>
+  </si>
+  <si>
+    <t>Routage entre frontend et microservices corrigé.</t>
+  </si>
+  <si>
+    <t>Données pour jeux, utilisateurs et posts ajoutées.</t>
+  </si>
+  <si>
+    <t>Navigation et structure du panneau admin améliorées.</t>
+  </si>
+  <si>
+    <t>J’ai ajouté des fichiers du chatbot</t>
+  </si>
+  <si>
+    <t>Images et assets du chatbot ajoutés.</t>
+  </si>
+  <si>
+    <t>J’ai amélioré le thème du site</t>
+  </si>
+  <si>
+    <t>Thèmes dynamiques et styles améliorés.</t>
+  </si>
+  <si>
+    <t>J’ai ajouté des personnages AI</t>
+  </si>
+  <si>
+    <t>Personas AI dynamiques ajoutés au chatbot.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,11 +258,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -182,16 +269,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -523,169 +610,390 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76940CD4-5DAD-4279-81E7-FE78E5A50C44}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="13.8"/>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.69921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="27.6">
-      <c r="A2" s="1">
+    <row r="2" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
         <v>46034</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="4">
         <v>0.58333333333333337</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="27.6">
-      <c r="A3" s="1">
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
         <v>46034</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="4">
         <v>0.61805555555555558</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="27.6">
-      <c r="A4" s="1">
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
         <v>46034</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="4">
         <v>0.65277777777777779</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="27.6">
-      <c r="A5" s="1">
+    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
         <v>46034</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="4">
         <v>0.6875</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="27.6">
-      <c r="A6" s="1">
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
         <v>46034</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <v>0.72916666666666663</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="41.4">
-      <c r="A7" s="1">
+    <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
         <v>46034</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="4">
         <v>0.77083333333333337</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>46327</v>
+      </c>
+      <c r="B8" s="4">
+        <v>0.8125</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="4">
+        <v>0.4375</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add male.jpg image to pixel assets
</commit_message>
<xml_diff>
--- a/docs/logbook.xlsx
+++ b/docs/logbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\01_Projects\EPITA\RetroHub\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A25E1FFA-9E51-454B-AE45-987180FA3284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BADB800-E234-4B5B-8373-8901A277C2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{8F73FF81-C54F-4E0C-9038-545D5E42BA1D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37710" windowHeight="21840" xr2:uid="{8F73FF81-C54F-4E0C-9038-545D5E42BA1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -20,21 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="52">
   <si>
     <t>Date</t>
   </si>
@@ -104,13 +95,112 @@
     <t>Documentation principale terminée.
 Toutes les tâches sont finies.
 Les tests ne sont pas encore faits.</t>
+  </si>
+  <si>
+    <t>J’ai ajouté Docker et MongoDB</t>
+  </si>
+  <si>
+    <t>14/01/2026</t>
+  </si>
+  <si>
+    <t>15/01/2026</t>
+  </si>
+  <si>
+    <t>J’ai amélioré le style du site</t>
+  </si>
+  <si>
+    <t>16/01/2026</t>
+  </si>
+  <si>
+    <t>J’ai conteneurisé l’application</t>
+  </si>
+  <si>
+    <t>Application complète lancée avec Docker.</t>
+  </si>
+  <si>
+    <t>17/01/2026</t>
+  </si>
+  <si>
+    <t>J’ai corrigé le proxy API</t>
+  </si>
+  <si>
+    <t>19/01/2026</t>
+  </si>
+  <si>
+    <t>J’ai ajouté des données de test</t>
+  </si>
+  <si>
+    <t>J’ai amélioré le panneau admin</t>
+  </si>
+  <si>
+    <t>20/01/2026</t>
+  </si>
+  <si>
+    <t>21/01/2026</t>
+  </si>
+  <si>
+    <t>Docker Compose configuré avec MongoDB et Mongo Express.</t>
+  </si>
+  <si>
+    <t>J’ai amélioré la base de données</t>
+  </si>
+  <si>
+    <t>Vérifications de connexion MongoDB ajoutées. Scripts Docker améliorés.</t>
+  </si>
+  <si>
+    <t>J’ai créé le logbook du projet</t>
+  </si>
+  <si>
+    <t>Fichier logbook ajouté et structuré.</t>
+  </si>
+  <si>
+    <t>J’ai amélioré l’interface admin</t>
+  </si>
+  <si>
+    <t>Gestion des erreurs et formulaires améliorés.</t>
+  </si>
+  <si>
+    <t>Thème, header et navigation mis à jour.</t>
+  </si>
+  <si>
+    <t>J’ai intégré le chat AI</t>
+  </si>
+  <si>
+    <t>Fonctionnalité de chat AI ajoutée au projet.</t>
+  </si>
+  <si>
+    <t>Routage entre frontend et microservices corrigé.</t>
+  </si>
+  <si>
+    <t>Données pour jeux, utilisateurs et posts ajoutées.</t>
+  </si>
+  <si>
+    <t>Navigation et structure du panneau admin améliorées.</t>
+  </si>
+  <si>
+    <t>J’ai ajouté des fichiers du chatbot</t>
+  </si>
+  <si>
+    <t>Images et assets du chatbot ajoutés.</t>
+  </si>
+  <si>
+    <t>J’ai amélioré le thème du site</t>
+  </si>
+  <si>
+    <t>Thèmes dynamiques et styles améliorés.</t>
+  </si>
+  <si>
+    <t>J’ai ajouté des personnages AI</t>
+  </si>
+  <si>
+    <t>Personas AI dynamiques ajoutés au chatbot.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,11 +258,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -182,16 +269,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -523,169 +610,390 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76940CD4-5DAD-4279-81E7-FE78E5A50C44}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="13.8"/>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.69921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="27.6">
-      <c r="A2" s="1">
+    <row r="2" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
         <v>46034</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="4">
         <v>0.58333333333333337</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="27.6">
-      <c r="A3" s="1">
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
         <v>46034</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="4">
         <v>0.61805555555555558</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="27.6">
-      <c r="A4" s="1">
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
         <v>46034</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="4">
         <v>0.65277777777777779</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="27.6">
-      <c r="A5" s="1">
+    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
         <v>46034</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="4">
         <v>0.6875</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="27.6">
-      <c r="A6" s="1">
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
         <v>46034</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <v>0.72916666666666663</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="41.4">
-      <c r="A7" s="1">
+    <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
         <v>46034</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="4">
         <v>0.77083333333333337</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="1"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>46327</v>
+      </c>
+      <c r="B8" s="4">
+        <v>0.8125</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="4">
+        <v>0.4375</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>